<commit_message>
feat: populate missing fields from annuaire and derive SIREN from SIRET
- Derive SIREN automatically from first 9 digits of SIRET when SIREN
  column is absent or blank, so SIRET-only rows are not skipped
- After a successful API lookup, fill any blank customer fields
  (Nom, SIRET, Code postal, Ville) from the annuaire response —
  compare() runs first so only originally-supplied values flag discrepancies
- Auto-populated cells highlighted in blue in the Excel report
- New "Source SIREN" column shows whether SIREN came from the file or
  was derived from SIRET
- New "Champs complétés" column lists fields auto-filled per row
- New Légende sheet explains all colour codes including blue
- Updated sample generator to include SIRET-only and partial-data rows

https://claude.ai/code/session_01LLgY3dAYjCq49wxWMHoofD
</commit_message>
<xml_diff>
--- a/annuaire-matcher/customers_sample.xlsx
+++ b/annuaire-matcher/customers_sample.xlsx
@@ -510,41 +510,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>542107651</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>54210765100015</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Société Générale</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>29 boulevard Haussmann</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>75009</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>factures@socgen.com</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,31 +528,15 @@
           <t>380129866</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>38012986600020</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Carrefour SA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>93 avenue de Paris</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>91300</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Massy</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>einvoice@carrefour.com</t>
@@ -605,25 +565,17 @@
           <t>69002</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Lyon</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>000000001</t>
+          <t>572073396</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SIREN invalide test</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>

</xml_diff>